<commit_message>
data: actualizacion automatica 2026-07-31
</commit_message>
<xml_diff>
--- a/data/estadisticas_poblacion_2026-07-31.xlsx
+++ b/data/estadisticas_poblacion_2026-07-31.xlsx
@@ -456,7 +456,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-31 15:18 UTC</t>
+          <t>2026-07-31 15:56 UTC</t>
         </is>
       </c>
     </row>
@@ -949,12 +949,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa (IDA &amp; IBRD countries)</t>
+          <t>Sub-Saharan Africa</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>TSS</t>
+          <t>SSF</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -970,12 +970,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa</t>
+          <t>Sub-Saharan Africa (IDA &amp; IBRD countries)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SSF</t>
+          <t>TSS</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -43857,12 +43857,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Sint Maarten (Dutch part)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>BMU</t>
+          <t>SXM</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -43872,21 +43872,21 @@
         <v>100</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.1</v>
+        <v>1.4</v>
       </c>
       <c r="F2" t="n">
-        <v>-5</v>
+        <v>558</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bahrain</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BHR</t>
+          <t>SGP</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -43896,21 +43896,21 @@
         <v>100</v>
       </c>
       <c r="E3" t="n">
-        <v>0.73</v>
+        <v>1.99</v>
       </c>
       <c r="F3" t="n">
-        <v>22699</v>
+        <v>20011</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sint Maarten (Dutch part)</t>
+          <t>Cayman Islands</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SXM</t>
+          <t>CYM</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -43920,21 +43920,21 @@
         <v>100</v>
       </c>
       <c r="E4" t="n">
-        <v>1.4</v>
+        <v>1.92</v>
       </c>
       <c r="F4" t="n">
-        <v>558</v>
+        <v>896</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Naoero</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SGP</t>
+          <t>NRU</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -43944,21 +43944,21 @@
         <v>100</v>
       </c>
       <c r="E5" t="n">
-        <v>1.99</v>
+        <v>0.6</v>
       </c>
       <c r="F5" t="n">
-        <v>20011</v>
+        <v>-121</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Naoero</t>
+          <t>Hong Kong SAR, China</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>NRU</t>
+          <t>HKG</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -43968,21 +43968,21 @@
         <v>100</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6</v>
+        <v>-0.16</v>
       </c>
       <c r="F6" t="n">
-        <v>-121</v>
+        <v>-19272</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kuwait</t>
+          <t>Bahrain</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KWT</t>
+          <t>BHR</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -43992,21 +43992,21 @@
         <v>100</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9</v>
+        <v>0.73</v>
       </c>
       <c r="F7" t="n">
-        <v>61624</v>
+        <v>22699</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Macao SAR, China</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MAC</t>
+          <t>BMU</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -44016,21 +44016,21 @@
         <v>100</v>
       </c>
       <c r="E8" t="n">
-        <v>1.2</v>
+        <v>-0.1</v>
       </c>
       <c r="F8" t="n">
-        <v>1620</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>St. Martin (French part)</t>
+          <t>Macao SAR, China</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MAF</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -44040,21 +44040,21 @@
         <v>100</v>
       </c>
       <c r="E9" t="n">
-        <v>-5.17</v>
+        <v>1.2</v>
       </c>
       <c r="F9" t="n">
-        <v>-1424</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Monaco</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MCO</t>
+          <t>KWT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -44064,21 +44064,21 @@
         <v>100</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.84</v>
+        <v>0.9</v>
       </c>
       <c r="F10" t="n">
-        <v>110</v>
+        <v>61624</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hong Kong SAR, China</t>
+          <t>Monaco</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HKG</t>
+          <t>MCO</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -44088,21 +44088,21 @@
         <v>100</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.16</v>
+        <v>-0.84</v>
       </c>
       <c r="F11" t="n">
-        <v>-19272</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Gibraltar</t>
+          <t>St. Martin (French part)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>GIB</t>
+          <t>MAF</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -44112,21 +44112,21 @@
         <v>100</v>
       </c>
       <c r="E12" t="n">
-        <v>2.21</v>
+        <v>-5.17</v>
       </c>
       <c r="F12" t="n">
-        <v>598</v>
+        <v>-1424</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cayman Islands</t>
+          <t>Gibraltar</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CYM</t>
+          <t>GIB</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -44136,10 +44136,10 @@
         <v>100</v>
       </c>
       <c r="E13" t="n">
-        <v>1.92</v>
+        <v>2.21</v>
       </c>
       <c r="F13" t="n">
-        <v>896</v>
+        <v>598</v>
       </c>
     </row>
     <row r="14">
@@ -49257,12 +49257,12 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>South Asia</t>
+          <t>South Asia (IDA &amp; IBRD)</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>SAS</t>
+          <t>TSA</t>
         </is>
       </c>
       <c r="C227" t="n">
@@ -49281,12 +49281,12 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>South Asia (IDA &amp; IBRD)</t>
+          <t>South Asia</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>TSA</t>
+          <t>SAS</t>
         </is>
       </c>
       <c r="C228" t="n">

</xml_diff>